<commit_message>
Update with new devices for the secondary side
</commit_message>
<xml_diff>
--- a/Switch Functions/Sec Data.xlsx
+++ b/Switch Functions/Sec Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Github\Switch Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F76918-952F-4D28-9313-1FB5FF8D89F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C24CF5-7A01-4299-9E7B-AE3E862CFDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1068,6 +1068,12 @@
       <c r="J11" s="2">
         <v>150</v>
       </c>
+      <c r="K11" s="6">
+        <v>1.28</v>
+      </c>
+      <c r="L11" s="6">
+        <v>2.14</v>
+      </c>
       <c r="M11" s="2">
         <v>20</v>
       </c>
@@ -1104,8 +1110,12 @@
       <c r="J12" s="2">
         <v>150</v>
       </c>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
+      <c r="K12" s="6">
+        <v>2.88</v>
+      </c>
+      <c r="L12" s="6">
+        <v>4.8099999999999996</v>
+      </c>
       <c r="M12" s="2">
         <v>22</v>
       </c>
@@ -1145,6 +1155,12 @@
       <c r="J13" s="2">
         <v>150</v>
       </c>
+      <c r="K13" s="6">
+        <v>1.65</v>
+      </c>
+      <c r="L13" s="6">
+        <v>2.08</v>
+      </c>
       <c r="M13" s="2">
         <v>23</v>
       </c>
@@ -1185,6 +1201,12 @@
       </c>
       <c r="J14" s="2">
         <v>150</v>
+      </c>
+      <c r="K14" s="6">
+        <v>1.83</v>
+      </c>
+      <c r="L14" s="6">
+        <v>2.02</v>
       </c>
       <c r="M14" s="2">
         <v>13</v>

</xml_diff>